<commit_message>
Sprint tracker: per-task DoD text and status updates
DoD column rewritten to be specific to each individual task instead of
one sentence duplicated across every task in a PBI. Status updated to
Done for T3.1-T3.4, T4.1-T4.4, and T6.1-T6.3, each verified against
real (non-mocked) API calls before being marked complete.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sprint_Tracker.xlsx
+++ b/Sprint_Tracker.xlsx
@@ -640,7 +640,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>spec.md, plan.md, tasks.md exist; plan.md resolves every open question; tasks.md is granular enough to execute; stakeholder signed off.</t>
+          <t>spec.md exists and clearly states the user story, what's in scope, what's out of scope, and the exact numbers that count as a successful test run.</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>spec.md, plan.md, tasks.md exist; plan.md resolves every open question; tasks.md is granular enough to execute; stakeholder signed off.</t>
+          <t>plan.md exists and every open design question has a real decision written down, not left blank.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>spec.md, plan.md, tasks.md exist; plan.md resolves every open question; tasks.md is granular enough to execute; stakeholder signed off.</t>
+          <t>tasks.md exists and breaks every PBI into small tasks specific enough that nobody has to ask 'what do you mean' before starting one.</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>spec.md, plan.md, tasks.md exist; plan.md resolves every open question; tasks.md is granular enough to execute; stakeholder signed off.</t>
+          <t>Someone has actually read spec.md, plan.md, and tasks.md and said 'yes, build this' - silence doesn't count as approval.</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Repo installs cleanly; lint passes; all schemas parse a sample JSON fixture each.</t>
+          <t>Running the install command works with no errors, and the linter (ruff) reports zero problems.</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Repo installs cleanly; lint passes; all schemas parse a sample JSON fixture each.</t>
+          <t>.env.example lists all three required keys (OpenRouter, Gemini, Groq) with no real secrets inside it, and the real .env file is excluded from git.</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Repo installs cleanly; lint passes; all schemas parse a sample JSON fixture each.</t>
+          <t>Every data shape from plan.md (EvalRun, LLMCallResult, etc.) exists as a schema, and each one can successfully load a small hand-written sample without crashing.</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Renderer produces a correctly filled prompt for every variant/test-case pair; missing-variable case caught with a readable error.</t>
+          <t>A real example JSON file exists with multiple prompt variants and test cases, and it loads successfully into the EvalRun schema with no errors.</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Renderer produces a correctly filled prompt for every variant/test-case pair; missing-variable case caught with a readable error.</t>
+          <t>Given one prompt variant and one test case, the renderer returns the template with every {blank} correctly replaced by the real value.</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Renderer produces a correctly filled prompt for every variant/test-case pair; missing-variable case caught with a readable error.</t>
+          <t>Tests exist and pass proving every variant/test-case combo renders correctly, and that a missing variable produces a clear, readable error instead of a raw crash.</t>
         </is>
       </c>
     </row>
@@ -1035,12 +1035,12 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>All N x M x K calls execute concurrently; every result is a valid LLMCallResult; a forced single-call failure doesn't abort the batch.</t>
+          <t>One function can send a prompt to any of the three providers (OpenRouter, Gemini, Groq) just by changing the model name string.</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>All N x M x K calls execute concurrently; every result is a valid LLMCallResult; a forced single-call failure doesn't abort the batch.</t>
+          <t>Multiple calls fire at the same time instead of one-by-one, and the number running at once never goes above the concurrency limit.</t>
         </is>
       </c>
     </row>
@@ -1115,12 +1115,12 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>All N x M x K calls execute concurrently; every result is a valid LLMCallResult; a forced single-call failure doesn't abort the batch.</t>
+          <t>Every successful call's result includes the real input token count, output token count, and how many milliseconds it took.</t>
         </is>
       </c>
     </row>
@@ -1155,12 +1155,12 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>All N x M x K calls execute concurrently; every result is a valid LLMCallResult; a forced single-call failure doesn't abort the batch.</t>
+          <t>A temporary failure (like a rate limit) gets retried automatically with increasing wait times; if it still fails after retries, the result's error field is filled in instead of the program crashing.</t>
         </is>
       </c>
     </row>
@@ -1195,12 +1195,12 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Every LLMCallResult gets a valid JudgeResult; a malformed judge response never raises past the retry/fallback path.</t>
+          <t>The judge prompt template exists and includes the rubric, the candidate answer, and clear instructions to return only JSON with a score and reasoning.</t>
         </is>
       </c>
     </row>
@@ -1235,12 +1235,12 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Every LLMCallResult gets a valid JudgeResult; a malformed judge response never raises past the retry/fallback path.</t>
+          <t>A real judge call returns a score from 1-5 plus reasoning text, and it loads correctly into the JudgeResult schema.</t>
         </is>
       </c>
     </row>
@@ -1275,12 +1275,12 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Every LLMCallResult gets a valid JudgeResult; a malformed judge response never raises past the retry/fallback path.</t>
+          <t>If the judge's response isn't valid JSON, the program asks again once; if it still fails, the result gets a score of 0 and a 'parse failure' reason instead of crashing.</t>
         </is>
       </c>
     </row>
@@ -1315,12 +1315,12 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Every LLMCallResult gets a valid JudgeResult; a malformed judge response never raises past the retry/fallback path.</t>
+          <t>Tests exist and pass for three cases: a valid JSON response, a broken JSON response, and a JSON response wrapped in markdown formatting.</t>
         </is>
       </c>
     </row>
@@ -1355,12 +1355,12 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>One end-to-end run produces a RunReport with a ranked table and a recommended_variant_id + rationale naming concrete reasons.</t>
+          <t>Each prompt variant gets one combined score built from its average quality, cost, and speed, using the weighting formula from plan.md.</t>
         </is>
       </c>
     </row>
@@ -1395,12 +1395,12 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>One end-to-end run produces a RunReport with a ranked table and a recommended_variant_id + rationale naming concrete reasons.</t>
+          <t>The program picks exactly one winning variant and writes a plain-English reason for why each other variant scored lower (quality, cost, or speed).</t>
         </is>
       </c>
     </row>
@@ -1435,12 +1435,12 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>One end-to-end run produces a RunReport with a ranked table and a recommended_variant_id + rationale naming concrete reasons.</t>
+          <t>Running a report prints a readable ranked table in the terminal and also saves the full results to a JSON file.</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Fresh clone + README-only setup produces a working run; no unhandled exceptions in the E2E pass.</t>
+          <t>Running the tool for real - 3 prompt variants x 5 test cases against all three providers - produces a complete report with no crashes.</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Fresh clone + README-only setup produces a working run; no unhandled exceptions in the E2E pass.</t>
+          <t>README.md lets someone install the tool, set up their API keys, and run their first evaluation using only the instructions in that file.</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Fresh clone + README-only setup produces a working run; no unhandled exceptions in the E2E pass.</t>
+          <t>Every issue found during the real end-to-end run in T8.1 has been fixed and re-tested.</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>cost_usd on a known token count matches a hand calculation; unknown models fall back to cost_usd=None.</t>
+          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>cost_usd on a known token count matches a hand calculation; unknown models fall back to cost_usd=None.</t>
+          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>A simulated timeout or mid-run failure still yields a RunReport containing every result that did complete.</t>
+          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>A simulated timeout or mid-run failure still yields a RunReport containing every result that did complete.</t>
+          <t>A call that hangs past the timeout limit gets cancelled and recorded as a timeout error, instead of hanging forever.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add interactive `prompteval init` setup wizard
New command that asks for the task name, prompt variants, test cases,
and judge rubric directly in the terminal instead of requiring a
hand-written JSON file, then saves the answers as a real EvalRun input
file ready for `prompteval run`.

Variable names ({placeholder} in a template) are inferred automatically
from whatever variants were entered, so every test case is prompted for
exactly the variables the templates actually need.

Not part of the original Tasks.md/Plan.md scope -- added on request.
Logged as PBI-10 in the sprint tracker for visibility.

Verified two ways: a scripted-answers test suite (tests/test_wizard.py,
tests/test_cli.py), and a real run piping answers into the actual
`prompteval init` command via stdin, then running the file it produced
through the real pipeline end-to-end.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sprint_Tracker.xlsx
+++ b/Sprint_Tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C5" s="4">
-        <f>SUM(E10:E39)</f>
+        <f>SUM(E10:E40)</f>
         <v/>
       </c>
     </row>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="C6" s="4">
-        <f>SUMIF(B10:B37,"Must",E10:E39)</f>
+        <f>SUMIF(B10:B37,"Must",E10:E40)</f>
         <v/>
       </c>
     </row>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>SUMIF(B10:B37,"Stretch",E10:E39)</f>
+        <f>SUMIF(B10:B37,"Stretch",E10:E40)</f>
         <v/>
       </c>
     </row>
@@ -1645,42 +1645,42 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>PBI-5 Cost &amp; Latency Calculation</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>T5.1</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Build pricing table ($ per input/output token)</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>Fri 7 Aug</t>
-        </is>
-      </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H36" s="8" t="inlineStr">
-        <is>
-          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PBI-10 Interactive Setup Wizard</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>T10.1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Add `prompteval init` -- asks for task name, prompt variants, test cases, and rubric in the terminal, then saves a real input file</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Tue 4 Aug</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Answering the terminal questions produces a real input file that `prompteval run` can load and execute with no manual edits needed.</t>
         </is>
       </c>
     </row>
@@ -1697,12 +1697,12 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Compute cost_usd per call/variant</t>
+          <t>Build pricing table ($ per input/output token)</t>
         </is>
       </c>
       <c r="E37" s="8" t="n">
@@ -1720,14 +1720,14 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
+          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>PBI-7 Error Handling &amp; Reliability</t>
+          <t>PBI-5 Cost &amp; Latency Calculation</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
@@ -1737,12 +1737,12 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T5.2</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Confirm partial failures never drop completed results</t>
+          <t>Compute cost_usd per call/variant</t>
         </is>
       </c>
       <c r="E38" s="8" t="n">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>Unscheduled (if time remains)</t>
+          <t>Fri 7 Aug</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
         </is>
       </c>
     </row>
@@ -1777,12 +1777,12 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>Add explicit per-provider timeout handling</t>
+          <t>Confirm partial failures never drop completed results</t>
         </is>
       </c>
       <c r="E39" s="8" t="n">
@@ -1799,6 +1799,46 @@
         </is>
       </c>
       <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>PBI-7 Error Handling &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>T7.2</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Add explicit per-provider timeout handling</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Unscheduled (if time remains)</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
         <is>
           <t>A call that hangs past the timeout limit gets cancelled and recorded as a timeout error, instead of hanging forever.</t>
         </is>

</xml_diff>

<commit_message>
Make quickstart the default when no subcommand is given
Running plain `prompteval` (or `prompteval --judge-model x` with only
flags, no subcommand) now runs the quickstart flow directly instead of
erroring out demanding a subcommand. `prompteval run <file>` and
`prompteval init` are unaffected -- routing only kicks in when argv[0]
isn't already a known subcommand.

Verified live: `prompteval --judge-model groq/llama-3.3-70b-versatile`
with no subcommand ran a full real quickstart evaluation end-to-end.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sprint_Tracker.xlsx
+++ b/Sprint_Tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C5" s="4">
-        <f>SUM(E10:E41)</f>
+        <f>SUM(E10:E42)</f>
         <v/>
       </c>
     </row>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="C6" s="4">
-        <f>SUMIF(B10:B37,"Must",E10:E41)</f>
+        <f>SUMIF(B10:B37,"Must",E10:E42)</f>
         <v/>
       </c>
     </row>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>SUMIF(B10:B37,"Stretch",E10:E41)</f>
+        <f>SUMIF(B10:B37,"Stretch",E10:E42)</f>
         <v/>
       </c>
     </row>
@@ -1725,42 +1725,42 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>PBI-5 Cost &amp; Latency Calculation</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>T5.1</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Build pricing table ($ per input/output token)</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>Fri 7 Aug</t>
-        </is>
-      </c>
-      <c r="G38" s="8" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H38" s="8" t="inlineStr">
-        <is>
-          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PBI-11 AI-Generated Quickstart</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>T11.2</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Make quickstart the default when `prompteval` is run with no subcommand (or only flags)</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Tue 4 Aug</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Typing plain 'prompteval' (or 'prompteval --judge-model x') with no subcommand at all starts the quickstart flow directly; 'prompteval run &lt;file&gt;' and 'prompteval init' still work exactly as before.</t>
         </is>
       </c>
     </row>
@@ -1777,12 +1777,12 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>Compute cost_usd per call/variant</t>
+          <t>Build pricing table ($ per input/output token)</t>
         </is>
       </c>
       <c r="E39" s="8" t="n">
@@ -1800,14 +1800,14 @@
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
+          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>PBI-7 Error Handling &amp; Reliability</t>
+          <t>PBI-5 Cost &amp; Latency Calculation</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
@@ -1817,12 +1817,12 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T5.2</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>Confirm partial failures never drop completed results</t>
+          <t>Compute cost_usd per call/variant</t>
         </is>
       </c>
       <c r="E40" s="8" t="n">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>Unscheduled (if time remains)</t>
+          <t>Fri 7 Aug</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1857,12 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Add explicit per-provider timeout handling</t>
+          <t>Confirm partial failures never drop completed results</t>
         </is>
       </c>
       <c r="E41" s="8" t="n">
@@ -1879,6 +1879,46 @@
         </is>
       </c>
       <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>PBI-7 Error Handling &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>T7.2</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Add explicit per-provider timeout handling</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>Unscheduled (if time remains)</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
         <is>
           <t>A call that hangs past the timeout limit gets cancelled and recorded as a timeout error, instead of hanging forever.</t>
         </is>

</xml_diff>

<commit_message>
Change the no-subcommand default from quickstart to improve
Bare `prompteval` (and the double-click Run PromtEval.cmd, which just
calls it with no subcommand) now goes straight into `improve` -- ask
for one prompt, get a score + rewrite -- instead of `quickstart`'s
3-prompt comparison flow. That turned out to be the actually-wanted
default; `quickstart`/`init`/`run` are unaffected when named explicitly.

Updated /help text and README to lead with `improve` as the default,
moved the multi-prompt-comparison commands (`quickstart`/`init`) to a
secondary section.

Verified live twice: bare `prompteval` and double-clicking the .cmd
button both produced a real score + rewritten prompt on the first
question asked, no subcommand typed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sprint_Tracker.xlsx
+++ b/Sprint_Tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C5" s="4">
-        <f>SUM(E10:E46)</f>
+        <f>SUM(E10:E47)</f>
         <v/>
       </c>
     </row>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="C6" s="4">
-        <f>SUMIF(B10:B37,"Must",E10:E46)</f>
+        <f>SUMIF(B10:B37,"Must",E10:E47)</f>
         <v/>
       </c>
     </row>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>SUMIF(B10:B37,"Stretch",E10:E46)</f>
+        <f>SUMIF(B10:B37,"Stretch",E10:E47)</f>
         <v/>
       </c>
     </row>
@@ -1925,42 +1925,42 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>PBI-5 Cost &amp; Latency Calculation</t>
-        </is>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>T5.1</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Build pricing table ($ per input/output token)</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>Fri 7 Aug</t>
-        </is>
-      </c>
-      <c r="G43" s="8" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H43" s="8" t="inlineStr">
-        <is>
-          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>PBI-15 Change Default to Improve</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>T15.1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Change the no-subcommand default (bare 'prompteval' and the double-click .cmd) from quickstart to improve, since single-prompt scoring turned out to be the actually wanted default flow</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Wed 5 Aug</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Bare 'prompteval' and double-clicking 'Run PromtEval.cmd' both now go straight into the improve flow (asks for one prompt, returns score + rewrite) -- confirmed with two separate live runs. 'quickstart'/'init'/'run' still work unchanged when named explicitly.</t>
         </is>
       </c>
     </row>
@@ -1977,12 +1977,12 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>Compute cost_usd per call/variant</t>
+          <t>Build pricing table ($ per input/output token)</t>
         </is>
       </c>
       <c r="E44" s="8" t="n">
@@ -2000,14 +2000,14 @@
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
+          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>PBI-7 Error Handling &amp; Reliability</t>
+          <t>PBI-5 Cost &amp; Latency Calculation</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -2017,12 +2017,12 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T5.2</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Confirm partial failures never drop completed results</t>
+          <t>Compute cost_usd per call/variant</t>
         </is>
       </c>
       <c r="E45" s="8" t="n">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>Unscheduled (if time remains)</t>
+          <t>Fri 7 Aug</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
         </is>
       </c>
     </row>
@@ -2057,12 +2057,12 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>Add explicit per-provider timeout handling</t>
+          <t>Confirm partial failures never drop completed results</t>
         </is>
       </c>
       <c r="E46" s="8" t="n">
@@ -2079,6 +2079,46 @@
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>PBI-7 Error Handling &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>T7.2</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Add explicit per-provider timeout handling</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>Unscheduled (if time remains)</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
         <is>
           <t>A call that hangs past the timeout limit gets cancelled and recorded as a timeout error, instead of hanging forever.</t>
         </is>

</xml_diff>

<commit_message>
Fix stale SUMIF ranges in Sprint_Tracker.xlsx
The Must-have/Stretch hour total formulas (rows 6-7) were stuck at
B10:B37/E10:E37 while new PBI rows kept getting inserted above the
original stretch-goal rows, pushing T7.1/T7.2 outside that range.
Stretch hours was undercounting by 2h as a result (only counting
T5.1/T5.2, missing T7.1/T7.2). Row 5's SUM formula had correctly grown
to E10:E47 already; 6-7 just never got updated alongside it.

Fixed by computing the actual last row dynamically (ws.max_row) instead
of hand-tracking it across incremental edits, and verified against a
manual sum: Total 44h, Must 30.5h, Stretch 4h (was 2h).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sprint_Tracker.xlsx
+++ b/Sprint_Tracker.xlsx
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="C6" s="4">
-        <f>SUMIF(B10:B37,"Must",E10:E47)</f>
+        <f>SUMIF(B10:B47,"Must",E10:E47)</f>
         <v/>
       </c>
     </row>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>SUMIF(B10:B37,"Stretch",E10:E47)</f>
+        <f>SUMIF(B10:B47,"Stretch",E10:E47)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Make the menu self-explanatory, add real menu-specific help
User feedback on the new menu: "Build a reusable input file" and "Run
an existing input file" weren't clear, and picking "Help" just
repeated the whole install/API-key guide instead of explaining the
menu itself.

- Reworded all 4 main choices to be self-explanatory on their own:
  "Save a prompt comparison to a file for later (doesn't run yet)" /
  "Run a prompt comparison file you already have", etc.
- Added MENU_HELP_TEXT: a focused explanation of exactly what each
  option does, with a plain-English example, shown when Help is picked
  from the menu -- separate from the general /help guide (still
  reachable via a one-line pointer at the end).

Verified live via the Git Bash fallback menu: selecting Help now shows
the new focused text, confirmed readable end to end.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sprint_Tracker.xlsx
+++ b/Sprint_Tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C5" s="4">
-        <f>SUM(E10:E49)</f>
+        <f>SUM(E10:E50)</f>
         <v/>
       </c>
     </row>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="C6" s="4">
-        <f>SUMIF(B10:B49,"Must",E10:E49)</f>
+        <f>SUMIF(B10:B50,"Must",E10:E50)</f>
         <v/>
       </c>
     </row>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>SUMIF(B10:B49,"Stretch",E10:E49)</f>
+        <f>SUMIF(B10:B50,"Stretch",E10:E50)</f>
         <v/>
       </c>
     </row>
@@ -2045,42 +2045,42 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>PBI-5 Cost &amp; Latency Calculation</t>
-        </is>
-      </c>
-      <c r="B46" s="8" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>T5.1</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Build pricing table ($ per input/output token)</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="n">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>PBI-16 Interactive Terminal Menu</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>T16.3</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>User feedback: menu's Help option just repeated the generic /help install guide, not useful in context; 'Build a reusable input file'/'Run an existing input file' choices were unclear. Reworded all 4 main choices to be self-explanatory and added a menu-specific MENU_HELP_TEXT explaining exactly what each option does</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
         <v>1</v>
       </c>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>Fri 7 Aug</t>
-        </is>
-      </c>
-      <c r="G46" s="8" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H46" s="8" t="inlineStr">
-        <is>
-          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Thu 6 Aug</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Selecting Help from the real menu (confirmed live) now explains each option in plain terms with a concrete example, instead of repeating the install/API-key guide.</t>
         </is>
       </c>
     </row>
@@ -2097,12 +2097,12 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Compute cost_usd per call/variant</t>
+          <t>Build pricing table ($ per input/output token)</t>
         </is>
       </c>
       <c r="E47" s="8" t="n">
@@ -2120,14 +2120,14 @@
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
+          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>PBI-7 Error Handling &amp; Reliability</t>
+          <t>PBI-5 Cost &amp; Latency Calculation</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
@@ -2137,12 +2137,12 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T5.2</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>Confirm partial failures never drop completed results</t>
+          <t>Compute cost_usd per call/variant</t>
         </is>
       </c>
       <c r="E48" s="8" t="n">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>Unscheduled (if time remains)</t>
+          <t>Fri 7 Aug</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
         </is>
       </c>
     </row>
@@ -2177,12 +2177,12 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>Add explicit per-provider timeout handling</t>
+          <t>Confirm partial failures never drop completed results</t>
         </is>
       </c>
       <c r="E49" s="8" t="n">
@@ -2199,6 +2199,46 @@
         </is>
       </c>
       <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>PBI-7 Error Handling &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>T7.2</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Add explicit per-provider timeout handling</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Unscheduled (if time remains)</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
         <is>
           <t>A call that hangs past the timeout limit gets cancelled and recorded as a timeout error, instead of hanging forever.</t>
         </is>

</xml_diff>

<commit_message>
Add Anthropic/Claude as a supported provider
LiteLLM already routes anthropic/claude-* model strings with zero code
changes needed (same as OpenRouter/Gemini/Groq) -- the only real gap
was the "is any API key configured?" guard not knowing about
ANTHROPIC_API_KEY, which would have wrongly told a Claude-only user
"no key found." Fixed that, plus added it to .env.example, /help, and
the no-key message (with a clear note that Anthropic has no free tier,
unlike the other three).

Verified with a real key: litellm successfully authenticated a live
request to Claude (claude-sonnet-5) -- confirmed by reaching a genuine
billing error ("credit balance too low") rather than an auth error,
proving the wiring itself is correct. Actual generation is blocked by
the account needing a paid balance, not a code issue.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sprint_Tracker.xlsx
+++ b/Sprint_Tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C5" s="4">
-        <f>SUM(E10:E50)</f>
+        <f>SUM(E10:E51)</f>
         <v/>
       </c>
     </row>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="C6" s="4">
-        <f>SUMIF(B10:B50,"Must",E10:E50)</f>
+        <f>SUMIF(B10:B51,"Must",E10:E51)</f>
         <v/>
       </c>
     </row>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>SUMIF(B10:B50,"Stretch",E10:E50)</f>
+        <f>SUMIF(B10:B51,"Stretch",E10:E51)</f>
         <v/>
       </c>
     </row>
@@ -2085,42 +2085,42 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>PBI-5 Cost &amp; Latency Calculation</t>
-        </is>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>T5.1</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Build pricing table ($ per input/output token)</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="8" t="inlineStr">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PBI-17 Anthropic/Claude Provider Support</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>T17.1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Add ANTHROPIC_API_KEY to the 'is any key configured?' check, .env.example, and /help + no-key message -- LiteLLM already routes anthropic/claude-* model strings with no other code changes needed</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F47" t="inlineStr">
         <is>
           <t>Fri 7 Aug</t>
         </is>
       </c>
-      <c r="G47" s="8" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H47" s="8" t="inlineStr">
-        <is>
-          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>A real Anthropic key was added and litellm successfully authenticated a live request to Claude (proven -- reached a genuine billing error, not an auth error). Actual generation is blocked by the account having a zero credit balance, a billing issue on the user's Anthropic account, not a code gap; the wiring itself is confirmed correct.</t>
         </is>
       </c>
     </row>
@@ -2137,12 +2137,12 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>Compute cost_usd per call/variant</t>
+          <t>Build pricing table ($ per input/output token)</t>
         </is>
       </c>
       <c r="E48" s="8" t="n">
@@ -2160,14 +2160,14 @@
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
+          <t>A pricing table exists listing $ per input token and $ per output token for every in-scope model.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>PBI-7 Error Handling &amp; Reliability</t>
+          <t>PBI-5 Cost &amp; Latency Calculation</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -2177,12 +2177,12 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>T7.1</t>
+          <t>T5.2</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>Confirm partial failures never drop completed results</t>
+          <t>Compute cost_usd per call/variant</t>
         </is>
       </c>
       <c r="E49" s="8" t="n">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>Unscheduled (if time remains)</t>
+          <t>Fri 7 Aug</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+          <t>Given a call's real token counts, the calculated dollar cost matches what you'd get doing the multiplication by hand.</t>
         </is>
       </c>
     </row>
@@ -2217,12 +2217,12 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>T7.2</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>Add explicit per-provider timeout handling</t>
+          <t>Confirm partial failures never drop completed results</t>
         </is>
       </c>
       <c r="E50" s="8" t="n">
@@ -2239,6 +2239,46 @@
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>If some calls in a batch fail, the finished ones are still included in the final report - nothing gets thrown away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>PBI-7 Error Handling &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>T7.2</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Add explicit per-provider timeout handling</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>Unscheduled (if time remains)</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
         <is>
           <t>A call that hangs past the timeout limit gets cancelled and recorded as a timeout error, instead of hanging forever.</t>
         </is>

</xml_diff>